<commit_message>
fix sales summary export
</commit_message>
<xml_diff>
--- a/uploads/excel/bulk_upload_sales_merge.xlsx
+++ b/uploads/excel/bulk_upload_sales_merge.xlsx
@@ -1,80 +1,73 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Glenn\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Henne\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12015" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="12">
+  <si>
+    <t>Reference Number</t>
+  </si>
+  <si>
+    <t>Settlement ID</t>
+  </si>
   <si>
     <t>Billing ID</t>
   </si>
   <si>
-    <t>Notes:</t>
-  </si>
-  <si>
-    <t>Make sure that the data in this sheet does not have any formula, values only</t>
-  </si>
-  <si>
-    <t>Do not move any rows and columns, just fill it out.</t>
-  </si>
-  <si>
     <t>Invoice Number</t>
   </si>
   <si>
-    <t xml:space="preserve">                                                                                                                                                                                                                                                                                                                                                                                                                                                               </t>
-  </si>
-  <si>
-    <t xml:space="preserve">                                         </t>
+    <t>TS-WF-219F-0030024</t>
   </si>
   <si>
     <t>1590EC</t>
   </si>
   <si>
-    <t>Reference Number</t>
-  </si>
-  <si>
-    <t>TS-WF-219F-0030024</t>
-  </si>
-  <si>
-    <t>Settlement ID</t>
+    <t>Reference No</t>
+  </si>
+  <si>
+    <t>TS-WF-234F-0050149</t>
+  </si>
+  <si>
+    <t>sales_merge_transaction_head</t>
+  </si>
+  <si>
+    <t>sales_merge_transaction_details</t>
+  </si>
+  <si>
+    <t>checker</t>
+  </si>
+  <si>
+    <t>to update if checker exist</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -92,29 +85,30 @@
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
+      <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -129,14 +123,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -171,7 +164,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -183,7 +176,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>
@@ -200,9 +193,9 @@
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -230,31 +223,14 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -282,23 +258,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -451,76 +410,117 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.5703125" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>8</v>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2">
+        <v>5</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="4">
         <v>1001</v>
-      </c>
-      <c r="H2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="E10" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="K16" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="E32:G36"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="32" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E32" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="F32" t="s">
+        <v>8</v>
+      </c>
+      <c r="G32" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E33" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E34" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+      <c r="G34" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E35" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+      <c r="G35" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E36" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+      <c r="G36" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>